<commit_message>
Kijelző-NYÁK (Rev. A) első élesztése: 8 MB flash; napló
- sdkconfig.defaults: 8 MB flash. A NYÁK modulja N8R8; a 16 MB-os
  beállítással az alkalmazás indításkor leállt (újraindulási hurok).
  A devkiten (N16R8) a 8 MB-os beállítás is fut.
- Napló: H-29 (flashméret), V-42 (a NYÁK élesztése: 3,3 V, PSRAM,
  kijelző 40 MHz-en, érintés és gesztusok rendben), Q-36 megválaszolva
  (a J2-n nincs felcserélve a két reset), új: Q-39 (a TP4056 LED-árama).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fejlesztesi_naplo.xlsx
+++ b/docs/fejlesztesi_naplo.xlsx
@@ -2569,7 +2569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="17" min="1" max="1"/>
@@ -4219,6 +4219,63 @@
       <c r="K29" s="27" t="inlineStr">
         <is>
           <t>esp_lvgl_port_touch.c</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="23.25" customHeight="1" s="18">
+      <c r="A30" s="27" t="inlineStr">
+        <is>
+          <t>H-29</t>
+        </is>
+      </c>
+      <c r="B30" s="27" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="C30" s="27" t="inlineStr">
+        <is>
+          <t>Display NYÁK (szoftver)</t>
+        </is>
+      </c>
+      <c r="D30" s="27" t="inlineStr">
+        <is>
+          <t>A display_node 16 MB-os flashre volt beállítva (fejlesztőpanel N16R8), a NYÁK modulja N8R8 (8 MB): az alkalmazás indításkor leállt ('Detected size(8192k) smaller than the size in the binary image header(16384k)'), és újraindulási hurokba került.</t>
+        </is>
+      </c>
+      <c r="E30" s="27" t="inlineStr">
+        <is>
+          <t>Soros napló a NYÁK első flashelésekor</t>
+        </is>
+      </c>
+      <c r="F30" s="27" t="inlineStr">
+        <is>
+          <t>Közepes</t>
+        </is>
+      </c>
+      <c r="G30" s="27" t="inlineStr">
+        <is>
+          <t>A NYÁK-on egyetlen alkalmazás sem indult el.</t>
+        </is>
+      </c>
+      <c r="H30" s="27" t="inlineStr">
+        <is>
+          <t>sdkconfig.defaults: 8 MB flash (a devkiten is fut); a NYÁK-hoz a menuconfigban a Rev. A lábkiosztás választandó.</t>
+        </is>
+      </c>
+      <c r="I30" s="27" t="inlineStr">
+        <is>
+          <t>V-42</t>
+        </is>
+      </c>
+      <c r="J30" s="27" t="inlineStr">
+        <is>
+          <t>Lezárva</t>
+        </is>
+      </c>
+      <c r="K30" s="27" t="inlineStr">
+        <is>
+          <t>firmware/display_node/sdkconfig.defaults</t>
         </is>
       </c>
     </row>
@@ -4246,7 +4303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="17" min="1" max="1"/>
@@ -6014,6 +6071,48 @@
         </is>
       </c>
       <c r="H42" s="27" t="inlineStr">
+        <is>
+          <t>Végrehajtva</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="46.25" customHeight="1" s="18">
+      <c r="A43" s="27" t="inlineStr">
+        <is>
+          <t>V-42</t>
+        </is>
+      </c>
+      <c r="B43" s="27" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="C43" s="27" t="inlineStr">
+        <is>
+          <t>Hardver / szoftver</t>
+        </is>
+      </c>
+      <c r="D43" s="27" t="inlineStr">
+        <is>
+          <t>A kijelző-NYÁK (Rev. A) első élesztése: 3,3 V a modulon (mérve), 8 MB Octal PSRAM rendben, ST77916 40 MHz-en zaj- és szaggatásmentes kép, CST816T (0xB5) érintés és gesztusok működnek; a flashméret 8 MB-ra állítva.</t>
+        </is>
+      </c>
+      <c r="E43" s="27" t="inlineStr">
+        <is>
+          <t>Megérkezett NYÁK-ok</t>
+        </is>
+      </c>
+      <c r="F43" s="27" t="inlineStr">
+        <is>
+          <t>H-29, Q-36</t>
+        </is>
+      </c>
+      <c r="G43" s="27" t="inlineStr">
+        <is>
+          <t>a lezáró commit</t>
+        </is>
+      </c>
+      <c r="H43" s="27" t="inlineStr">
         <is>
           <t>Végrehajtva</t>
         </is>
@@ -6832,7 +6931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="17" min="1" max="1"/>
@@ -7827,7 +7926,7 @@
       </c>
       <c r="C37" s="27" t="inlineStr">
         <is>
-          <t>A saját NYÁK J2 csatlakozóján is fel van-e cserélve a kijelző és az érintő resetje (mint a modul 15 pólusú csatlakozóján, H-27)?</t>
+          <t>A saját NYÁK J2 csatlakozóján is fel van-e cserélve a kijelző és az érintő resetje (mint a modul 15 pólusú csatlakozóján, H-27)? Válasz (2026-10-27): nem; a NYÁK-on az érintőt az IO14 (TP_RST) ébreszti, a kijelző resetje (IO45) nem altatja el. A felcserélés csak a modul 15 pólusú csatlakozóján van, a Rev. A lábkiosztás jó.</t>
         </is>
       </c>
       <c r="D37" s="27" t="inlineStr">
@@ -7837,7 +7936,7 @@
       </c>
       <c r="E37" s="27" t="inlineStr">
         <is>
-          <t>Nyitott</t>
+          <t>Megválaszolt</t>
         </is>
       </c>
     </row>
@@ -7890,6 +7989,33 @@
         </is>
       </c>
       <c r="E39" s="27" t="inlineStr">
+        <is>
+          <t>Nyitott</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="23.25" customHeight="1" s="18">
+      <c r="A40" s="27" t="inlineStr">
+        <is>
+          <t>Q-39</t>
+        </is>
+      </c>
+      <c r="B40" s="27" t="inlineStr">
+        <is>
+          <t>Display NYÁK</t>
+        </is>
+      </c>
+      <c r="C40" s="27" t="inlineStr">
+        <is>
+          <t>A TP4056 zöld (STDBY) LED-je 1 kOhm-mal nagyon erősen világít: a becslés szerint 2–3 mA, ami a határértékeken belül van; mérendő az ellenálláson eső feszültséggel, és akkumulátorral a CHRG/STDBY váltás is ellenőrizendő.</t>
+        </is>
+      </c>
+      <c r="D40" s="27" t="inlineStr">
+        <is>
+          <t>Feszültségmérés az 1 kOhm-on; töltésteszt LiPo-val</t>
+        </is>
+      </c>
+      <c r="E40" s="27" t="inlineStr">
         <is>
           <t>Nyitott</t>
         </is>

</xml_diff>